<commit_message>
Add basic info in doc files
</commit_message>
<xml_diff>
--- a/Week_1/HTTP 5310 – Capstone Timesheet_Ripal Patel.xlsx
+++ b/Week_1/HTTP 5310 – Capstone Timesheet_Ripal Patel.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="HTTP-5310-HTTP-5310Capstone_Tim" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="HTTP-5310- Capstone_Timesheet" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Week_1</t>
   </si>
@@ -34,13 +34,31 @@
     <t>Tech Stack choices</t>
   </si>
   <si>
-    <t>Theme + Create Github Repo</t>
+    <t>Create Github Repo + ReadMe file</t>
+  </si>
+  <si>
+    <t>Work on website Theme</t>
+  </si>
+  <si>
+    <t>Finalize Theme + colors + typography</t>
+  </si>
+  <si>
+    <t>Requirements Document</t>
+  </si>
+  <si>
+    <t>Timeline</t>
+  </si>
+  <si>
+    <t>Technical Barriers Assessment Doc file</t>
+  </si>
+  <si>
+    <t>Work on User Stories</t>
+  </si>
+  <si>
+    <t>Create Basic Wireframes for all the pages</t>
   </si>
   <si>
     <t>Total</t>
-  </si>
-  <si>
-    <t>Total Hours</t>
   </si>
 </sst>
 </file>
@@ -80,7 +98,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -97,12 +115,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFC27BA0"/>
         <bgColor rgb="FFC27BA0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA64D79"/>
-        <bgColor rgb="FFA64D79"/>
       </patternFill>
     </fill>
   </fills>
@@ -126,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -150,15 +162,6 @@
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
   </cellXfs>
@@ -379,7 +382,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="10.0"/>
-    <col customWidth="1" min="2" max="2" width="45.38"/>
+    <col customWidth="1" min="2" max="2" width="47.75"/>
     <col customWidth="1" min="3" max="3" width="12.25"/>
     <col customWidth="1" min="4" max="4" width="12.13"/>
   </cols>
@@ -500,7 +503,7 @@
         <v>46037.0</v>
       </c>
       <c r="D4" s="4">
-        <v>1.5</v>
+        <v>2.0</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
@@ -535,7 +538,7 @@
         <v>46037.0</v>
       </c>
       <c r="D5" s="4">
-        <v>2.0</v>
+        <v>1.15</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -562,14 +565,15 @@
       <c r="AA5" s="3"/>
     </row>
     <row r="6">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7" t="s">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="7">
-        <f>sum(D2:D5)</f>
-        <v>4.95</v>
+      <c r="C6" s="5">
+        <v>46038.0</v>
+      </c>
+      <c r="D6" s="4">
+        <v>4.75</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -596,10 +600,16 @@
       <c r="AA6" s="3"/>
     </row>
     <row r="7">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
+      <c r="A7" s="4"/>
+      <c r="B7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="5">
+        <v>46038.0</v>
+      </c>
+      <c r="D7" s="4">
+        <v>3.5</v>
+      </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="3"/>
@@ -625,10 +635,16 @@
       <c r="AA7" s="3"/>
     </row>
     <row r="8">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
+      <c r="A8" s="4"/>
+      <c r="B8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="5">
+        <v>46038.0</v>
+      </c>
+      <c r="D8" s="4">
+        <v>5.75</v>
+      </c>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="3"/>
@@ -654,10 +670,16 @@
       <c r="AA8" s="3"/>
     </row>
     <row r="9">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
+      <c r="A9" s="4"/>
+      <c r="B9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="5">
+        <v>46039.0</v>
+      </c>
+      <c r="D9" s="4">
+        <v>3.0</v>
+      </c>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="3"/>
@@ -683,14 +705,15 @@
       <c r="AA9" s="3"/>
     </row>
     <row r="10">
-      <c r="A10" s="9"/>
-      <c r="B10" s="10" t="s">
-        <v>9</v>
+      <c r="A10" s="4"/>
+      <c r="B10" s="4" t="s">
+        <v>12</v>
       </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="10">
-        <f>sum(D2:D5)</f>
-        <v>4.95</v>
+      <c r="C10" s="5">
+        <v>46039.0</v>
+      </c>
+      <c r="D10" s="4">
+        <v>5.5</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -717,12 +740,18 @@
       <c r="AA10" s="3"/>
     </row>
     <row r="11">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
+      <c r="A11" s="4"/>
+      <c r="B11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="5">
+        <v>46041.0</v>
+      </c>
+      <c r="D11" s="4">
+        <v>4.75</v>
+      </c>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -746,12 +775,18 @@
       <c r="AA11" s="3"/>
     </row>
     <row r="12">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
+      <c r="A12" s="4"/>
+      <c r="B12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="5">
+        <v>46043.0</v>
+      </c>
+      <c r="D12" s="4">
+        <v>4.75</v>
+      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
@@ -775,12 +810,17 @@
       <c r="AA12" s="3"/>
     </row>
     <row r="13">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
+      <c r="A13" s="7"/>
+      <c r="B13" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="8"/>
+      <c r="D13" s="7">
+        <f>sum(D2:D12)</f>
+        <v>36.6</v>
+      </c>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
@@ -804,12 +844,12 @@
       <c r="AA13" s="3"/>
     </row>
     <row r="14">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
@@ -833,12 +873,12 @@
       <c r="AA14" s="3"/>
     </row>
     <row r="15">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
@@ -862,12 +902,12 @@
       <c r="AA15" s="3"/>
     </row>
     <row r="16">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
@@ -891,12 +931,8 @@
       <c r="AA16" s="3"/>
     </row>
     <row r="17">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
@@ -28324,64 +28360,6 @@
       <c r="Z962" s="3"/>
       <c r="AA962" s="3"/>
     </row>
-    <row r="963">
-      <c r="A963" s="3"/>
-      <c r="B963" s="3"/>
-      <c r="C963" s="3"/>
-      <c r="D963" s="3"/>
-      <c r="E963" s="3"/>
-      <c r="F963" s="3"/>
-      <c r="G963" s="3"/>
-      <c r="H963" s="3"/>
-      <c r="I963" s="3"/>
-      <c r="J963" s="3"/>
-      <c r="K963" s="3"/>
-      <c r="L963" s="3"/>
-      <c r="M963" s="3"/>
-      <c r="N963" s="3"/>
-      <c r="O963" s="3"/>
-      <c r="P963" s="3"/>
-      <c r="Q963" s="3"/>
-      <c r="R963" s="3"/>
-      <c r="S963" s="3"/>
-      <c r="T963" s="3"/>
-      <c r="U963" s="3"/>
-      <c r="V963" s="3"/>
-      <c r="W963" s="3"/>
-      <c r="X963" s="3"/>
-      <c r="Y963" s="3"/>
-      <c r="Z963" s="3"/>
-      <c r="AA963" s="3"/>
-    </row>
-    <row r="964">
-      <c r="A964" s="3"/>
-      <c r="B964" s="3"/>
-      <c r="C964" s="3"/>
-      <c r="D964" s="3"/>
-      <c r="E964" s="3"/>
-      <c r="F964" s="3"/>
-      <c r="G964" s="3"/>
-      <c r="H964" s="3"/>
-      <c r="I964" s="3"/>
-      <c r="J964" s="3"/>
-      <c r="K964" s="3"/>
-      <c r="L964" s="3"/>
-      <c r="M964" s="3"/>
-      <c r="N964" s="3"/>
-      <c r="O964" s="3"/>
-      <c r="P964" s="3"/>
-      <c r="Q964" s="3"/>
-      <c r="R964" s="3"/>
-      <c r="S964" s="3"/>
-      <c r="T964" s="3"/>
-      <c r="U964" s="3"/>
-      <c r="V964" s="3"/>
-      <c r="W964" s="3"/>
-      <c r="X964" s="3"/>
-      <c r="Y964" s="3"/>
-      <c r="Z964" s="3"/>
-      <c r="AA964" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Add User stories and update timesheet & Timeline
</commit_message>
<xml_diff>
--- a/Week_1/HTTP 5310 – Capstone Timesheet_Ripal Patel.xlsx
+++ b/Week_1/HTTP 5310 – Capstone Timesheet_Ripal Patel.xlsx
@@ -678,7 +678,7 @@
         <v>46039.0</v>
       </c>
       <c r="D9" s="4">
-        <v>3.0</v>
+        <v>5.0</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
@@ -810,15 +810,10 @@
       <c r="AA12" s="3"/>
     </row>
     <row r="13">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="7">
-        <f>sum(D2:D12)</f>
-        <v>36.6</v>
-      </c>
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="4"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
       <c r="G13" s="3"/>
@@ -844,10 +839,15 @@
       <c r="AA13" s="3"/>
     </row>
     <row r="14">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
+      <c r="A14" s="7"/>
+      <c r="B14" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="8"/>
+      <c r="D14" s="7">
+        <f>sum(D2:D12)</f>
+        <v>38.6</v>
+      </c>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="3"/>
@@ -931,6 +931,10 @@
       <c r="AA16" s="3"/>
     </row>
     <row r="17">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="3"/>
@@ -956,12 +960,8 @@
       <c r="AA17" s="3"/>
     </row>
     <row r="18">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
@@ -28360,6 +28360,35 @@
       <c r="Z962" s="3"/>
       <c r="AA962" s="3"/>
     </row>
+    <row r="963">
+      <c r="A963" s="3"/>
+      <c r="B963" s="3"/>
+      <c r="C963" s="3"/>
+      <c r="D963" s="3"/>
+      <c r="E963" s="3"/>
+      <c r="F963" s="3"/>
+      <c r="G963" s="3"/>
+      <c r="H963" s="3"/>
+      <c r="I963" s="3"/>
+      <c r="J963" s="3"/>
+      <c r="K963" s="3"/>
+      <c r="L963" s="3"/>
+      <c r="M963" s="3"/>
+      <c r="N963" s="3"/>
+      <c r="O963" s="3"/>
+      <c r="P963" s="3"/>
+      <c r="Q963" s="3"/>
+      <c r="R963" s="3"/>
+      <c r="S963" s="3"/>
+      <c r="T963" s="3"/>
+      <c r="U963" s="3"/>
+      <c r="V963" s="3"/>
+      <c r="W963" s="3"/>
+      <c r="X963" s="3"/>
+      <c r="Y963" s="3"/>
+      <c r="Z963" s="3"/>
+      <c r="AA963" s="3"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
adding Project Timline and Timesheet
</commit_message>
<xml_diff>
--- a/Week_1/HTTP 5310 – Capstone Timesheet_Ripal Patel.xlsx
+++ b/Week_1/HTTP 5310 – Capstone Timesheet_Ripal Patel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
   <si>
     <t>Week_1</t>
   </si>
@@ -60,13 +60,50 @@
   <si>
     <t>Total</t>
   </si>
+  <si>
+    <t>Week_2</t>
+  </si>
+  <si>
+    <t>Review wireframe feedback</t>
+  </si>
+  <si>
+    <t>Update wireframes</t>
+  </si>
+  <si>
+    <t>Finalize wireframes</t>
+  </si>
+  <si>
+    <t>Update feature list</t>
+  </si>
+  <si>
+    <t>Organize feature priorities</t>
+  </si>
+  <si>
+    <t>Review course critical path</t>
+  </si>
+  <si>
+    <t>Create project milestones</t>
+  </si>
+  <si>
+    <t>Finalize project timeline</t>
+  </si>
+  <si>
+    <t>Identify technical risks</t>
+  </si>
+  <si>
+    <t>Identify content risks</t>
+  </si>
+  <si>
+    <t>Write mitigation strategies</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd-mmm"/>
+    <numFmt numFmtId="165" formatCode="d-mmm"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -77,28 +114,27 @@
     </font>
     <font>
       <b/>
-      <sz val="16.0"/>
+      <sz val="14.0"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
     </font>
     <font>
-      <sz val="16.0"/>
+      <sz val="14.0"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
     </font>
     <font>
-      <sz val="16.0"/>
+      <sz val="14.0"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="16.0"/>
+      <sz val="14.0"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -115,6 +151,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFC27BA0"/>
         <bgColor rgb="FFC27BA0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D2E9"/>
+        <bgColor rgb="FFD9D2E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB4A7D6"/>
+        <bgColor rgb="FFB4A7D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -138,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="17">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -162,6 +210,26 @@
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
   </cellXfs>
@@ -931,10 +999,18 @@
       <c r="AA16" s="3"/>
     </row>
     <row r="17">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
+      <c r="A17" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>3</v>
+      </c>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="3"/>
@@ -960,6 +1036,16 @@
       <c r="AA17" s="3"/>
     </row>
     <row r="18">
+      <c r="A18" s="10"/>
+      <c r="B18" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" s="12">
+        <v>46044.0</v>
+      </c>
+      <c r="D18" s="13">
+        <v>1.5</v>
+      </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="3"/>
@@ -985,10 +1071,16 @@
       <c r="AA18" s="3"/>
     </row>
     <row r="19">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
+      <c r="A19" s="10"/>
+      <c r="B19" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="12">
+        <v>46044.0</v>
+      </c>
+      <c r="D19" s="13">
+        <v>2.0</v>
+      </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
@@ -1014,10 +1106,16 @@
       <c r="AA19" s="3"/>
     </row>
     <row r="20">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
+      <c r="A20" s="10"/>
+      <c r="B20" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" s="12">
+        <v>46044.0</v>
+      </c>
+      <c r="D20" s="13">
+        <v>2.0</v>
+      </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -1043,10 +1141,16 @@
       <c r="AA20" s="3"/>
     </row>
     <row r="21">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
+      <c r="A21" s="10"/>
+      <c r="B21" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" s="12">
+        <v>46045.0</v>
+      </c>
+      <c r="D21" s="13">
+        <v>2.0</v>
+      </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
@@ -1072,10 +1176,16 @@
       <c r="AA21" s="3"/>
     </row>
     <row r="22">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
+      <c r="A22" s="10"/>
+      <c r="B22" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="12">
+        <v>46045.0</v>
+      </c>
+      <c r="D22" s="13">
+        <v>2.0</v>
+      </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -1101,10 +1211,16 @@
       <c r="AA22" s="3"/>
     </row>
     <row r="23">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
+      <c r="A23" s="10"/>
+      <c r="B23" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" s="12">
+        <v>46046.0</v>
+      </c>
+      <c r="D23" s="13">
+        <v>1.5</v>
+      </c>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
@@ -1130,10 +1246,16 @@
       <c r="AA23" s="3"/>
     </row>
     <row r="24">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
+      <c r="A24" s="10"/>
+      <c r="B24" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C24" s="12">
+        <v>46046.0</v>
+      </c>
+      <c r="D24" s="13">
+        <v>2.0</v>
+      </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
@@ -1159,10 +1281,16 @@
       <c r="AA24" s="3"/>
     </row>
     <row r="25">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
+      <c r="A25" s="10"/>
+      <c r="B25" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" s="12">
+        <v>46046.0</v>
+      </c>
+      <c r="D25" s="13">
+        <v>2.0</v>
+      </c>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
@@ -1188,10 +1316,16 @@
       <c r="AA25" s="3"/>
     </row>
     <row r="26">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
+      <c r="A26" s="10"/>
+      <c r="B26" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26" s="12">
+        <v>46047.0</v>
+      </c>
+      <c r="D26" s="13">
+        <v>2.0</v>
+      </c>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
@@ -1217,10 +1351,16 @@
       <c r="AA26" s="3"/>
     </row>
     <row r="27">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
+      <c r="A27" s="10"/>
+      <c r="B27" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" s="12">
+        <v>46047.0</v>
+      </c>
+      <c r="D27" s="13">
+        <v>2.0</v>
+      </c>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
@@ -1246,10 +1386,16 @@
       <c r="AA27" s="3"/>
     </row>
     <row r="28">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
+      <c r="A28" s="10"/>
+      <c r="B28" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" s="12">
+        <v>46047.0</v>
+      </c>
+      <c r="D28" s="13">
+        <v>2.0</v>
+      </c>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
@@ -1275,10 +1421,10 @@
       <c r="AA28" s="3"/>
     </row>
     <row r="29">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
+      <c r="A29" s="14"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
@@ -1304,10 +1450,10 @@
       <c r="AA29" s="3"/>
     </row>
     <row r="30">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
@@ -1333,10 +1479,10 @@
       <c r="AA30" s="3"/>
     </row>
     <row r="31">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
+      <c r="A31" s="14"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
@@ -1362,12 +1508,17 @@
       <c r="AA31" s="3"/>
     </row>
     <row r="32">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
+      <c r="A32" s="15"/>
+      <c r="B32" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C32" s="16"/>
+      <c r="D32" s="15">
+        <f>sum(D20:D30)</f>
+        <v>17.5</v>
+      </c>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>

</xml_diff>